<commit_message>
Digital Products lane: US-first (dollars, US fees and law, US English)
</commit_message>
<xml_diff>
--- a/resources/digital-products/files/dp-adv-cac-ceiling.xlsx
+++ b/resources/digital-products/files/dp-adv-cac-ceiling.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="£#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="$#,##0.00"/>
   </numFmts>
   <fonts count="12">
     <font>
@@ -532,7 +532,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -578,7 +578,7 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Average order value (£)</t>
+          <t>Average order value ($)</t>
         </is>
       </c>
       <c r="B6" s="7" t="n">
@@ -613,7 +613,7 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Cost per visitor from ads (£)</t>
+          <t>Cost per visitor from ads ($)</t>
         </is>
       </c>
       <c r="B9" s="7" t="n">
@@ -640,7 +640,7 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Contribution per order (£)</t>
+          <t>Contribution per order ($)</t>
         </is>
       </c>
       <c r="B13" s="9">
@@ -651,7 +651,7 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Break-even CAC (£)</t>
+          <t>Break-even CAC ($)</t>
         </is>
       </c>
       <c r="B14" s="10">
@@ -667,7 +667,7 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Safe CAC ceiling (£)</t>
+          <t>Safe CAC ceiling ($)</t>
         </is>
       </c>
       <c r="B15" s="9">
@@ -683,7 +683,7 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>What a customer actually costs you (£)</t>
+          <t>What a customer actually costs you ($)</t>
         </is>
       </c>
       <c r="B16" s="9">
@@ -705,7 +705,7 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Book: contribution £41.14; 70% → £28.80 ceiling; ads at 40p / 1% = £40 → burning the buffer.</t>
+          <t>Book: contribution $41.14; 70% → $28.80 ceiling; ads at 40¢ / 1% = $40 → burning the buffer.</t>
         </is>
       </c>
     </row>
@@ -740,5 +740,6 @@
     <mergeCell ref="A23:C23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Footer line: ePORTS — your ecom source (eports.global)
</commit_message>
<xml_diff>
--- a/resources/digital-products/files/dp-adv-cac-ceiling.xlsx
+++ b/resources/digital-products/files/dp-adv-cac-ceiling.xlsx
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -568,6 +568,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
@@ -630,6 +631,7 @@
         <v>1</v>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
@@ -702,6 +704,7 @@
         <v/>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
@@ -716,6 +719,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="13" t="n"/>
       <c r="B22" s="13" t="n"/>
@@ -728,12 +732,17 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>ePORTS — your ecom source. eports.global.</t>
-        </is>
-      </c>
+          <t>ePORTS — your ecom source (eports.global)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26"/>
+    <row r="27">
+      <c r="A27" s="15" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>